<commit_message>
fix: update platemap.xlsx to match the csv version and add Experiment and Name columns.
</commit_message>
<xml_diff>
--- a/tests/test_data/platemap.xlsx
+++ b/tests/test_data/platemap.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/acjs/bnext/code/bnext/cdk/tests/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC9352BB-9FC6-F345-BA9E-21F1A849A29B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31FA969B-E7BE-814C-A388-AE8C2E656A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4120" yWindow="760" windowWidth="26320" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="45">
   <si>
     <t>Well</t>
   </si>
@@ -98,6 +98,63 @@
   </si>
   <si>
     <t>C8</t>
+  </si>
+  <si>
+    <t>Experiment</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Concentration</t>
+  </si>
+  <si>
+    <t>Artifact</t>
+  </si>
+  <si>
+    <t>pT7-deGFP 100</t>
+  </si>
+  <si>
+    <t>pT7-deGFP 50</t>
+  </si>
+  <si>
+    <t>pT7-deGFP 20</t>
+  </si>
+  <si>
+    <t>pT7-deGFP 10</t>
+  </si>
+  <si>
+    <t>pT7-deGFP 5</t>
+  </si>
+  <si>
+    <t>pT7-deGFP 2</t>
+  </si>
+  <si>
+    <t>pT7-deGFP 1</t>
+  </si>
+  <si>
+    <t>pT7-deGFP 0</t>
+  </si>
+  <si>
+    <t>pT7-lacO-plamGFP 29.3</t>
+  </si>
+  <si>
+    <t>pT7-lacO-plamGFP 35.8</t>
+  </si>
+  <si>
+    <t>pT7-lacO-plamGFP 17.1</t>
+  </si>
+  <si>
+    <t>pT7-tetO-plamGFP 72.7</t>
+  </si>
+  <si>
+    <t>pT7-tetO-plamGFP 46.4</t>
+  </si>
+  <si>
+    <t>pT7-tetO-plamGFP 12.3</t>
+  </si>
+  <si>
+    <t>pT7-deGFP 178.5</t>
   </si>
 </sst>
 </file>
@@ -383,201 +440,305 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="4.1640625" customWidth="1"/>
-    <col min="2" max="2" width="29.83203125" customWidth="1"/>
-    <col min="3" max="5" width="28.33203125" customWidth="1"/>
-    <col min="6" max="6" width="9.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.33203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.5" customWidth="1"/>
+    <col min="4" max="4" width="29.83203125" customWidth="1"/>
+    <col min="5" max="7" width="28.33203125" customWidth="1"/>
+    <col min="8" max="8" width="9.83203125" customWidth="1"/>
+    <col min="9" max="9" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="2"/>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1">
+      <c r="B2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="B3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1">
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1">
+      <c r="B5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1">
+      <c r="B6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1">
+      <c r="B7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C9" s="1">
+      <c r="B9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="1">
+      <c r="E10" s="1">
         <v>29.3</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="1">
+      <c r="E11" s="1">
         <v>35.799999999999997</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="1">
+      <c r="E12" s="1">
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="1">
+      <c r="E13" s="1">
         <v>72.7</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="1">
+      <c r="E14" s="1">
         <v>46.4</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="1">
+      <c r="E15" s="1">
         <v>12.3</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C16" s="1">
+      <c r="B16" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E16" s="1">
         <v>178.5</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1">
+      <c r="B17" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" s="1">
         <v>178.5</v>
       </c>
     </row>

</xml_diff>